<commit_message>
v17.7 sheet v82 re-exported with the shortened yant words and the window's hint
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012dssR6qAN57acivr6t6QeS
</commit_message>
<xml_diff>
--- a/masters/v17.7/masterz-text-v82.xlsx
+++ b/masters/v17.7/masterz-text-v82.xlsx
@@ -5408,7 +5408,7 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t xml:space="preserve">The Nine Spires: the nine peaks of Mount Meru, home of the gods, and the nine qualities of the Buddha, each spire crowned with the three ovals that stand for him. Inked at the top of the back, it protects against weapons, danger, evil spirits and black magic. A Sak Yant is for life: it cannot be taken off.</t>
+          <t xml:space="preserve">The Nine Spires: the nine peaks of Mount Meru, home of the gods, and the nine qualities of the Buddha, each spire crowned with the three ovals that stand for him. Inked at the top of the back, it protects against weapons, danger, evil spirits and black magic.</t>
         </is>
       </c>
     </row>
@@ -5459,7 +5459,7 @@
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t xml:space="preserve">The Five Rows with the Diamond Canopy. Each row is a blessing: protection of the home, help through bad luck, protection from black magic and spirits, good fortune and success, and Metta Mahaniyom, loving kindness and charisma. The Chat Petch adds prosperity and support through difficult periods. A Sak Yant is for life: it cannot be taken off.</t>
+          <t xml:space="preserve">The Five Rows with the Diamond Canopy. Each row is a blessing: protection of the home, help through bad luck, protection from black magic and spirits, good fortune and success, and Metta Mahaniyom, loving kindness and charisma. The Chat Petch adds prosperity and support through difficult periods.</t>
         </is>
       </c>
     </row>
@@ -5510,7 +5510,7 @@
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t xml:space="preserve">A sacred ornament of script worn like a necklace, close to the body. For prosperity, good luck and protection, the strength to overcome obstacles, charm and respect, and a sense of security and inner power. A Sak Yant is for life: it cannot be taken off.</t>
+          <t xml:space="preserve">A sacred ornament of script worn like a necklace, close to the body. For prosperity, good luck and protection, the strength to overcome obstacles, charm and respect, and a sense of security and inner power.</t>
         </is>
       </c>
     </row>
@@ -11694,7 +11694,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">e3c1.A.text</t>
+          <t xml:space="preserve">e3c1.words.yantHint</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -11704,14 +11704,14 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Luck. For my business."</t>
+          <t xml:space="preserve">A Sak Yant is for life and cannot be taken off. Pick one, then confirm.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">e3c1.A.say</t>
+          <t xml:space="preserve">e3c1.A.text</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -11721,14 +11721,14 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t xml:space="preserve">I asked for luck. He told me what it would cost.</t>
+          <t xml:space="preserve">"Luck. For my business."</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">e3c1.A.teach</t>
+          <t xml:space="preserve">e3c1.A.say</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -11738,14 +11738,14 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Luck is a fine reason to begin. It is a poor reason to stay.</t>
+          <t xml:space="preserve">I asked for luck. He told me what it would cost.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">e3c1.B.text</t>
+          <t xml:space="preserve">e3c1.A.teach</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -11755,14 +11755,14 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Protection. From whatever's out there."</t>
+          <t xml:space="preserve">Luck is a fine reason to begin. It is a poor reason to stay.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">e3c1.B.say</t>
+          <t xml:space="preserve">e3c1.B.text</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -11772,14 +11772,14 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t xml:space="preserve">I asked for protection. He pointed at my own chest.</t>
+          <t xml:space="preserve">"Protection. From whatever's out there."</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">e3c1.B.teach</t>
+          <t xml:space="preserve">e3c1.B.say</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -11789,14 +11789,14 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Protection from outside begins with what you carry inside.</t>
+          <t xml:space="preserve">I asked for protection. He pointed at my own chest.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">e3c1.C.text</t>
+          <t xml:space="preserve">e3c1.B.teach</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -11806,14 +11806,14 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Next time, give me the strongest one you have."</t>
+          <t xml:space="preserve">Protection from outside begins with what you carry inside.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">e3c1.C.say</t>
+          <t xml:space="preserve">e3c1.C.text</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -11823,14 +11823,14 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t xml:space="preserve">I asked for more. He showed me I hadn't understood the first.</t>
+          <t xml:space="preserve">"Next time, give me the strongest one you have."</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">e3c1.C.teach</t>
+          <t xml:space="preserve">e3c1.C.say</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -11840,14 +11840,14 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wanting the strongest is wanting a power you have not yet earned the understanding of.</t>
+          <t xml:space="preserve">I asked for more. He showed me I hadn't understood the first.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">e3c1.D.text</t>
+          <t xml:space="preserve">e3c1.C.teach</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -11857,14 +11857,14 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t xml:space="preserve">"What does it ask of me?"</t>
+          <t xml:space="preserve">Wanting the strongest is wanting a power you have not yet earned the understanding of.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">e3c1.D.say</t>
+          <t xml:space="preserve">e3c1.D.text</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -11874,22 +11874,39 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t xml:space="preserve">I asked what it wanted from me. That was the right question.</t>
+          <t xml:space="preserve">"What does it ask of me?"</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
+          <t xml:space="preserve">e3c1.D.say</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EPISODE 3 · CHAPTER 1 — the story itself</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">I asked what it wanted from me. That was the right question.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
           <t xml:space="preserve">e3c1.D.teach</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="B47" t="inlineStr">
         <is>
           <t xml:space="preserve">EPISODE 3 · CHAPTER 1 — the story itself</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C47" t="inlineStr">
         <is>
           <t xml:space="preserve">Before you ask what a practice will give you, ask what it will ask of you.</t>
         </is>

</xml_diff>